<commit_message>
feat: last update bofl
</commit_message>
<xml_diff>
--- a/Sale_Order_Size (2).xlsx
+++ b/Sale_Order_Size (2).xlsx
@@ -148,31 +148,31 @@
     <t>46#</t>
   </si>
   <si>
-    <t>15E09A9042</t>
-  </si>
-  <si>
-    <t>15F09A9042</t>
-  </si>
-  <si>
-    <t>15G09A9042</t>
-  </si>
-  <si>
-    <t>15H09A9042</t>
-  </si>
-  <si>
-    <t>15I09A9042</t>
-  </si>
-  <si>
-    <t>15J09A9042</t>
-  </si>
-  <si>
-    <t>15K09A9042</t>
-  </si>
-  <si>
-    <t>15L09A9042</t>
-  </si>
-  <si>
-    <t>15M09A9042</t>
+    <t>15E09A9125</t>
+  </si>
+  <si>
+    <t>15F09A9125</t>
+  </si>
+  <si>
+    <t>15G09A9125</t>
+  </si>
+  <si>
+    <t>15H09A9125</t>
+  </si>
+  <si>
+    <t>15I09A9125</t>
+  </si>
+  <si>
+    <t>15J09A9125</t>
+  </si>
+  <si>
+    <t>15K09A9125</t>
+  </si>
+  <si>
+    <t>15L09A9125</t>
+  </si>
+  <si>
+    <t>15M09A9125</t>
   </si>
 </sst>
 </file>
@@ -757,13 +757,13 @@
         <v>43</v>
       </c>
       <c r="B3" s="6">
-        <v>100</v>
+        <v>33</v>
       </c>
       <c r="C3" s="6">
-        <v>100</v>
+        <v>34</v>
       </c>
       <c r="D3" s="6">
-        <v>100</v>
+        <v>33</v>
       </c>
       <c r="E3" s="6"/>
       <c r="F3" s="6"/>

</xml_diff>

<commit_message>
sample sheet to production sheet
</commit_message>
<xml_diff>
--- a/Sale_Order_Size (2).xlsx
+++ b/Sale_Order_Size (2).xlsx
@@ -148,31 +148,31 @@
     <t>46#</t>
   </si>
   <si>
-    <t>15E09A9125</t>
-  </si>
-  <si>
-    <t>15F09A9125</t>
-  </si>
-  <si>
-    <t>15G09A9125</t>
-  </si>
-  <si>
-    <t>15H09A9125</t>
-  </si>
-  <si>
-    <t>15I09A9125</t>
-  </si>
-  <si>
-    <t>15J09A9125</t>
-  </si>
-  <si>
-    <t>15K09A9125</t>
-  </si>
-  <si>
-    <t>15L09A9125</t>
-  </si>
-  <si>
-    <t>15M09A9125</t>
+    <t>15E09A9153</t>
+  </si>
+  <si>
+    <t>15F09A9153</t>
+  </si>
+  <si>
+    <t>15G09A9153</t>
+  </si>
+  <si>
+    <t>15H09A9153</t>
+  </si>
+  <si>
+    <t>15I09A9153</t>
+  </si>
+  <si>
+    <t>15J09A9153</t>
+  </si>
+  <si>
+    <t>15K09A9153</t>
+  </si>
+  <si>
+    <t>15L09A9153</t>
+  </si>
+  <si>
+    <t>15M09A9153</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
export flow is done
</commit_message>
<xml_diff>
--- a/Sale_Order_Size (2).xlsx
+++ b/Sale_Order_Size (2).xlsx
@@ -148,31 +148,31 @@
     <t>46#</t>
   </si>
   <si>
-    <t>15E09A9153</t>
-  </si>
-  <si>
-    <t>15F09A9153</t>
-  </si>
-  <si>
-    <t>15G09A9153</t>
-  </si>
-  <si>
-    <t>15H09A9153</t>
-  </si>
-  <si>
-    <t>15I09A9153</t>
-  </si>
-  <si>
-    <t>15J09A9153</t>
-  </si>
-  <si>
-    <t>15K09A9153</t>
-  </si>
-  <si>
-    <t>15L09A9153</t>
-  </si>
-  <si>
-    <t>15M09A9153</t>
+    <t>15E09A9176</t>
+  </si>
+  <si>
+    <t>15F09A9176</t>
+  </si>
+  <si>
+    <t>15G09A9176</t>
+  </si>
+  <si>
+    <t>15H09A9176</t>
+  </si>
+  <si>
+    <t>15I09A9176</t>
+  </si>
+  <si>
+    <t>15J09A9176</t>
+  </si>
+  <si>
+    <t>15K09A9176</t>
+  </si>
+  <si>
+    <t>15L09A9176</t>
+  </si>
+  <si>
+    <t>15M09A9176</t>
   </si>
 </sst>
 </file>

</xml_diff>